<commit_message>
Update analysis scripts, gitignore, and tables; archive old models/tables
</commit_message>
<xml_diff>
--- a/output/tables/Tables.xlsx
+++ b/output/tables/Tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ostatemailokstate-my.sharepoint.com/personal/tanner_scholten_okstate_edu/Documents/Thesis Project/Data/R/output/tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="11_B70A9E09FFC9B723F6CC1CB4DBEE4E05C67F1CA0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74AB699D-A6B6-44FD-A972-DF5DD79E12F1}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="11_B70A9E09FFC9B723F6CC1CB4DBEE4E05C67F1CA0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4EAF925D-81C0-4D4D-8DDE-F8C6C819ED03}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="20970" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-83" yWindow="0" windowWidth="10965" windowHeight="12233" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Species List" sheetId="1" r:id="rId1"/>
@@ -951,7 +951,7 @@
       <numFmt numFmtId="165" formatCode="#,##0.0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="#,##0.0"/>
+      <numFmt numFmtId="164" formatCode="#,##0.000"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="165" formatCode="#,##0.0"/>
@@ -963,7 +963,7 @@
       <numFmt numFmtId="165" formatCode="#,##0.0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="#,##0.000"/>
+      <numFmt numFmtId="165" formatCode="#,##0.0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1081,12 +1081,12 @@
   <autoFilter ref="A1:G16" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Assemblage"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Samples (n)" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Samples (n)" dataDxfId="13"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Method"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="SC"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="qD" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="qD.LCL" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0300-000007000000}" name="qD.UCL" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="qD" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="qD.LCL" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0300-000007000000}" name="qD.UCL" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1099,7 +1099,7 @@
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Assemblage"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Number of Samples"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="Observed Richness"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="Estimated Sample Coverage" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="Estimated Sample Coverage" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1163,10 +1163,10 @@
   <autoFilter ref="A1:E8" xr:uid="{00000000-0009-0000-0100-000009000000}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0800-000001000000}" name="Site"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0800-000002000000}" name="Cast Net" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0800-000003000000}" name="Centipede Net" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0800-000004000000}" name="Seine" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0800-000005000000}" name="All Gears" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0800-000002000000}" name="Cast Net" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0800-000003000000}" name="Centipede Net" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0800-000004000000}" name="Seine" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0800-000005000000}" name="All Gears" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1490,15 +1490,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E100"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="2" width="26.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="26.73046875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.73046875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1515,7 +1515,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -1532,7 +1532,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
@@ -1549,7 +1549,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
@@ -1566,7 +1566,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
@@ -1583,7 +1583,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
         <v>13</v>
       </c>
@@ -1600,7 +1600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
         <v>15</v>
       </c>
@@ -1617,7 +1617,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="s">
         <v>17</v>
       </c>
@@ -1634,7 +1634,7 @@
         <v>901</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
         <v>19</v>
       </c>
@@ -1651,7 +1651,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A10" s="2" t="s">
         <v>21</v>
       </c>
@@ -1668,7 +1668,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" s="2" t="s">
         <v>23</v>
       </c>
@@ -1685,7 +1685,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" s="2" t="s">
         <v>25</v>
       </c>
@@ -1702,7 +1702,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A13" s="2" t="s">
         <v>27</v>
       </c>
@@ -1719,7 +1719,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A14" s="2" t="s">
         <v>29</v>
       </c>
@@ -1736,7 +1736,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A15" s="2" t="s">
         <v>31</v>
       </c>
@@ -1753,7 +1753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A16" s="2" t="s">
         <v>33</v>
       </c>
@@ -1770,7 +1770,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17" s="2" t="s">
         <v>35</v>
       </c>
@@ -1787,7 +1787,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A18" s="2" t="s">
         <v>37</v>
       </c>
@@ -1804,7 +1804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A19" s="2" t="s">
         <v>39</v>
       </c>
@@ -1821,7 +1821,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A20" s="2" t="s">
         <v>41</v>
       </c>
@@ -1838,7 +1838,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A21" s="2" t="s">
         <v>43</v>
       </c>
@@ -1855,7 +1855,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A22" s="2" t="s">
         <v>45</v>
       </c>
@@ -1872,7 +1872,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A23" s="2" t="s">
         <v>47</v>
       </c>
@@ -1889,7 +1889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A24" s="2" t="s">
         <v>49</v>
       </c>
@@ -1906,7 +1906,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A25" s="2" t="s">
         <v>51</v>
       </c>
@@ -1923,7 +1923,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A26" s="2" t="s">
         <v>53</v>
       </c>
@@ -1940,7 +1940,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A27" s="2" t="s">
         <v>55</v>
       </c>
@@ -1957,7 +1957,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A28" s="2" t="s">
         <v>57</v>
       </c>
@@ -1974,7 +1974,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A29" s="2" t="s">
         <v>59</v>
       </c>
@@ -1991,7 +1991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A30" s="2" t="s">
         <v>61</v>
       </c>
@@ -2008,7 +2008,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A31" s="2" t="s">
         <v>63</v>
       </c>
@@ -2025,7 +2025,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A32" s="2" t="s">
         <v>65</v>
       </c>
@@ -2042,7 +2042,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A33" s="2" t="s">
         <v>67</v>
       </c>
@@ -2059,7 +2059,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A34" s="2" t="s">
         <v>69</v>
       </c>
@@ -2076,7 +2076,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A35" s="2" t="s">
         <v>71</v>
       </c>
@@ -2093,7 +2093,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A36" s="2" t="s">
         <v>73</v>
       </c>
@@ -2110,7 +2110,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A37" s="2" t="s">
         <v>75</v>
       </c>
@@ -2127,7 +2127,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A38" s="2" t="s">
         <v>77</v>
       </c>
@@ -2144,7 +2144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A39" s="2" t="s">
         <v>79</v>
       </c>
@@ -2161,7 +2161,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A40" s="2" t="s">
         <v>81</v>
       </c>
@@ -2178,7 +2178,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A41" s="2" t="s">
         <v>83</v>
       </c>
@@ -2195,7 +2195,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A42" s="2" t="s">
         <v>85</v>
       </c>
@@ -2212,7 +2212,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A43" s="2" t="s">
         <v>87</v>
       </c>
@@ -2229,7 +2229,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A44" s="2" t="s">
         <v>89</v>
       </c>
@@ -2246,7 +2246,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A45" s="2" t="s">
         <v>91</v>
       </c>
@@ -2263,7 +2263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A46" s="2" t="s">
         <v>93</v>
       </c>
@@ -2280,7 +2280,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A47" s="2" t="s">
         <v>95</v>
       </c>
@@ -2297,7 +2297,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A48" s="2" t="s">
         <v>97</v>
       </c>
@@ -2314,7 +2314,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A49" s="2" t="s">
         <v>99</v>
       </c>
@@ -2331,7 +2331,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A50" s="2" t="s">
         <v>101</v>
       </c>
@@ -2348,7 +2348,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A51" s="2" t="s">
         <v>103</v>
       </c>
@@ -2365,7 +2365,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A52" s="2" t="s">
         <v>105</v>
       </c>
@@ -2382,7 +2382,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A53" s="2" t="s">
         <v>107</v>
       </c>
@@ -2399,7 +2399,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A54" s="2" t="s">
         <v>109</v>
       </c>
@@ -2416,7 +2416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A55" s="2" t="s">
         <v>111</v>
       </c>
@@ -2433,7 +2433,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A56" s="2" t="s">
         <v>113</v>
       </c>
@@ -2450,7 +2450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A57" s="2" t="s">
         <v>115</v>
       </c>
@@ -2467,7 +2467,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A58" s="2" t="s">
         <v>117</v>
       </c>
@@ -2484,7 +2484,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A59" s="2" t="s">
         <v>119</v>
       </c>
@@ -2501,7 +2501,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A60" s="2" t="s">
         <v>121</v>
       </c>
@@ -2518,7 +2518,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A61" s="2" t="s">
         <v>123</v>
       </c>
@@ -2535,7 +2535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A62" s="2" t="s">
         <v>125</v>
       </c>
@@ -2552,7 +2552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A63" s="2" t="s">
         <v>127</v>
       </c>
@@ -2569,7 +2569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A64" s="2" t="s">
         <v>129</v>
       </c>
@@ -2586,7 +2586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A65" s="2" t="s">
         <v>131</v>
       </c>
@@ -2603,7 +2603,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A66" s="2" t="s">
         <v>133</v>
       </c>
@@ -2620,7 +2620,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A67" s="2" t="s">
         <v>135</v>
       </c>
@@ -2637,7 +2637,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A68" s="2" t="s">
         <v>137</v>
       </c>
@@ -2654,7 +2654,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A69" s="2" t="s">
         <v>139</v>
       </c>
@@ -2671,7 +2671,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A70" s="2" t="s">
         <v>141</v>
       </c>
@@ -2688,7 +2688,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A71" s="2" t="s">
         <v>143</v>
       </c>
@@ -2705,7 +2705,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A72" s="2" t="s">
         <v>145</v>
       </c>
@@ -2722,7 +2722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A73" s="2" t="s">
         <v>147</v>
       </c>
@@ -2739,7 +2739,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A74" s="2" t="s">
         <v>149</v>
       </c>
@@ -2756,7 +2756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A75" s="2" t="s">
         <v>151</v>
       </c>
@@ -2773,7 +2773,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A76" s="2" t="s">
         <v>153</v>
       </c>
@@ -2790,7 +2790,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A77" s="2" t="s">
         <v>155</v>
       </c>
@@ -2807,7 +2807,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A78" s="2" t="s">
         <v>157</v>
       </c>
@@ -2824,7 +2824,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A79" s="2" t="s">
         <v>159</v>
       </c>
@@ -2841,7 +2841,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A80" s="2" t="s">
         <v>161</v>
       </c>
@@ -2858,7 +2858,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A81" s="2" t="s">
         <v>163</v>
       </c>
@@ -2875,7 +2875,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A82" s="2" t="s">
         <v>165</v>
       </c>
@@ -2892,7 +2892,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A83" s="2" t="s">
         <v>167</v>
       </c>
@@ -2909,7 +2909,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A84" s="2" t="s">
         <v>169</v>
       </c>
@@ -2926,7 +2926,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A85" s="2" t="s">
         <v>171</v>
       </c>
@@ -2943,7 +2943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A86" s="2" t="s">
         <v>173</v>
       </c>
@@ -2960,7 +2960,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A87" s="2" t="s">
         <v>175</v>
       </c>
@@ -2977,7 +2977,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A88" s="2" t="s">
         <v>177</v>
       </c>
@@ -2994,73 +2994,73 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A89" s="3"/>
       <c r="C89" s="5"/>
       <c r="D89" s="5"/>
       <c r="E89" s="5"/>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A90" s="3"/>
       <c r="C90" s="5"/>
       <c r="D90" s="5"/>
       <c r="E90" s="5"/>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A91" s="3"/>
       <c r="C91" s="5"/>
       <c r="D91" s="5"/>
       <c r="E91" s="5"/>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A92" s="3"/>
       <c r="C92" s="5"/>
       <c r="D92" s="5"/>
       <c r="E92" s="5"/>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A93" s="3"/>
       <c r="C93" s="5"/>
       <c r="D93" s="5"/>
       <c r="E93" s="5"/>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A94" s="3"/>
       <c r="C94" s="5"/>
       <c r="D94" s="5"/>
       <c r="E94" s="5"/>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A95" s="3"/>
       <c r="C95" s="5"/>
       <c r="D95" s="5"/>
       <c r="E95" s="5"/>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A96" s="3"/>
       <c r="C96" s="5"/>
       <c r="D96" s="5"/>
       <c r="E96" s="5"/>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A97" s="3"/>
       <c r="C97" s="5"/>
       <c r="D97" s="5"/>
       <c r="E97" s="5"/>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A98" s="3"/>
       <c r="C98" s="5"/>
       <c r="D98" s="5"/>
       <c r="E98" s="5"/>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A99" s="3"/>
       <c r="C99" s="5"/>
       <c r="D99" s="5"/>
       <c r="E99" s="5"/>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A100" s="3"/>
       <c r="C100" s="5"/>
       <c r="D100" s="5"/>
@@ -3079,19 +3079,19 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="22.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.73046875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.73046875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.73046875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.73046875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.73046875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>254</v>
       </c>
@@ -3117,7 +3117,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>17</v>
       </c>
@@ -3143,7 +3143,7 @@
         <v>901</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>71</v>
       </c>
@@ -3169,7 +3169,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -3195,7 +3195,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>21</v>
       </c>
@@ -3221,7 +3221,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>111</v>
       </c>
@@ -3260,13 +3260,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="17.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.73046875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>258</v>
       </c>
@@ -3274,7 +3274,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>223</v>
       </c>
@@ -3282,7 +3282,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>259</v>
       </c>
@@ -3290,7 +3290,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>260</v>
       </c>
@@ -3298,7 +3298,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>261</v>
       </c>
@@ -3306,7 +3306,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>262</v>
       </c>
@@ -3314,7 +3314,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>263</v>
       </c>
@@ -3322,7 +3322,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>264</v>
       </c>
@@ -3343,17 +3343,17 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="25.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.73046875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.73046875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.73046875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -3373,7 +3373,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -3393,7 +3393,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
@@ -3413,7 +3413,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>67</v>
       </c>
@@ -3433,7 +3433,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>77</v>
       </c>
@@ -3453,7 +3453,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>79</v>
       </c>
@@ -3473,7 +3473,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>81</v>
       </c>
@@ -3493,7 +3493,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>117</v>
       </c>
@@ -3513,7 +3513,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>119</v>
       </c>
@@ -3533,7 +3533,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>125</v>
       </c>
@@ -3553,7 +3553,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>129</v>
       </c>
@@ -3573,7 +3573,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>149</v>
       </c>
@@ -3593,7 +3593,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>165</v>
       </c>
@@ -3613,7 +3613,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>171</v>
       </c>
@@ -3633,7 +3633,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>224</v>
       </c>
@@ -3653,7 +3653,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>224</v>
       </c>
@@ -3673,7 +3673,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>224</v>
       </c>
@@ -3693,7 +3693,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
         <v>224</v>
       </c>
@@ -3713,7 +3713,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
         <v>224</v>
       </c>
@@ -3733,7 +3733,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A20" s="1" t="s">
         <v>224</v>
       </c>
@@ -3766,17 +3766,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:M7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="9" width="16.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.73046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.73046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="9" width="16.73046875" bestFit="1" customWidth="1"/>
     <col min="10" max="11" width="15" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.7265625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.73046875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.73046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>179</v>
       </c>
@@ -3817,7 +3817,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>192</v>
       </c>
@@ -3858,7 +3858,7 @@
         <v>8.5624885294581699</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>194</v>
       </c>
@@ -3899,7 +3899,7 @@
         <v>9.4745502577614804</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>196</v>
       </c>
@@ -3940,7 +3940,7 @@
         <v>9.5863830295383892</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>197</v>
       </c>
@@ -3981,7 +3981,7 @@
         <v>5.5141788211503098</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>198</v>
       </c>
@@ -4022,7 +4022,7 @@
         <v>10.2978273919505</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>199</v>
       </c>
@@ -4076,17 +4076,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:J2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="17.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="8" width="18.7265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="28.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.73046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.73046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.73046875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="17.73046875" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="18.73046875" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="28.73046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>201</v>
       </c>
@@ -4118,7 +4118,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A2" s="1">
         <v>4372</v>
       </c>
@@ -4163,16 +4163,16 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:I16"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="24.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="16.7265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.73046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.73046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="15.73046875" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="16.73046875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>211</v>
       </c>
@@ -4195,7 +4195,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -4222,7 +4222,7 @@
         <v>37 (30.3, 43.6)</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -4249,7 +4249,7 @@
         <v>35.2 (30, 40.3)</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -4276,7 +4276,7 @@
         <v>30.9 (23.3, 38.6)</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>220</v>
       </c>
@@ -4303,7 +4303,7 @@
         <v>48.2 (41.8, 54.7)</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>221</v>
       </c>
@@ -4330,7 +4330,7 @@
         <v>41 (33.8, 48.3)</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>222</v>
       </c>
@@ -4357,7 +4357,7 @@
         <v>40.9 (35.1, 46.7)</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>223</v>
       </c>
@@ -4384,7 +4384,7 @@
         <v>48.6 (42.1, 55)</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>224</v>
       </c>
@@ -4407,7 +4407,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>2</v>
       </c>
@@ -4434,7 +4434,7 @@
         <v>56.2 (37.2, 75.1)</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>3</v>
       </c>
@@ -4461,7 +4461,7 @@
         <v>59.2 (45.4, 73)</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>4</v>
       </c>
@@ -4488,7 +4488,7 @@
         <v>67 (39.7, 94.3)</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>220</v>
       </c>
@@ -4515,7 +4515,7 @@
         <v>82.1 (67.2, 97)</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>221</v>
       </c>
@@ -4542,7 +4542,7 @@
         <v>81.9 (61.9, 101.8)</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>222</v>
       </c>
@@ -4569,7 +4569,7 @@
         <v>78.9 (63.1, 94.7)</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>223</v>
       </c>
@@ -4609,14 +4609,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="24.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="17.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.73046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="17.73046875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.73046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>211</v>
       </c>
@@ -4630,7 +4630,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -4644,7 +4644,7 @@
         <v>0.84360000000000002</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -4658,7 +4658,7 @@
         <v>0.90500000000000003</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -4672,7 +4672,7 @@
         <v>0.85850000000000004</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>220</v>
       </c>
@@ -4686,7 +4686,7 @@
         <v>0.9083</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>221</v>
       </c>
@@ -4700,7 +4700,7 @@
         <v>0.87970000000000004</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>222</v>
       </c>
@@ -4714,7 +4714,7 @@
         <v>0.91139999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>223</v>
       </c>
@@ -4741,14 +4741,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G26"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="24.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="7" width="16.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.73046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.73046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="7" width="16.73046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>211</v>
       </c>
@@ -4771,7 +4771,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -4794,7 +4794,7 @@
         <v>88.818621421860598</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -4817,7 +4817,7 @@
         <v>84.590625185324996</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -4840,7 +4840,7 @@
         <v>114.204362579158</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>220</v>
       </c>
@@ -4863,7 +4863,7 @@
         <v>112.358145476027</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>221</v>
       </c>
@@ -4886,7 +4886,7 @@
         <v>123.076028545536</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>222</v>
       </c>
@@ -4909,7 +4909,7 @@
         <v>111.233641006082</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>223</v>
       </c>
@@ -4932,7 +4932,7 @@
         <v>131.89053314338699</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>224</v>
       </c>
@@ -4955,7 +4955,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>2</v>
       </c>
@@ -4978,7 +4978,7 @@
         <v>47.801075992723597</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>3</v>
       </c>
@@ -5001,7 +5001,7 @@
         <v>44.921632371717998</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>4</v>
       </c>
@@ -5024,7 +5024,7 @@
         <v>41.685619744821899</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>220</v>
       </c>
@@ -5047,7 +5047,7 @@
         <v>61.460169643151097</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>221</v>
       </c>
@@ -5070,7 +5070,7 @@
         <v>53.263786068989099</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>222</v>
       </c>
@@ -5093,7 +5093,7 @@
         <v>54.750472020099302</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>223</v>
       </c>
@@ -5116,7 +5116,7 @@
         <v>62.610089026331501</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>224</v>
       </c>
@@ -5139,7 +5139,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
         <v>2</v>
       </c>
@@ -5162,7 +5162,7 @@
         <v>29.3545921123557</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
         <v>3</v>
       </c>
@@ -5185,7 +5185,7 @@
         <v>26.779764092876199</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A20" s="1" t="s">
         <v>4</v>
       </c>
@@ -5208,7 +5208,7 @@
         <v>24.073012752472501</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="7"/>
@@ -5217,7 +5217,7 @@
       <c r="F21" s="7"/>
       <c r="G21" s="7"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" s="1" t="s">
         <v>220</v>
       </c>
@@ -5240,7 +5240,7 @@
         <v>37.129045038812102</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" s="1" t="s">
         <v>221</v>
       </c>
@@ -5263,7 +5263,7 @@
         <v>29.934443283660599</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" s="1" t="s">
         <v>222</v>
       </c>
@@ -5286,7 +5286,7 @@
         <v>33.153843289340401</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="7"/>
@@ -5295,7 +5295,7 @@
       <c r="F25" s="7"/>
       <c r="G25" s="7"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" s="1" t="s">
         <v>223</v>
       </c>
@@ -5331,19 +5331,19 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:N8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="24.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="17.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="16.7265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="22.7265625" bestFit="1" customWidth="1"/>
-    <col min="11" max="13" width="16.7265625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.73046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="15.73046875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.73046875" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="17.73046875" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="16.73046875" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="22.73046875" bestFit="1" customWidth="1"/>
+    <col min="11" max="13" width="16.73046875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.73046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>239</v>
       </c>
@@ -5387,7 +5387,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -5431,7 +5431,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -5475,7 +5475,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -5519,7 +5519,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>220</v>
       </c>
@@ -5563,7 +5563,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>221</v>
       </c>
@@ -5607,7 +5607,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>222</v>
       </c>
@@ -5651,7 +5651,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>223</v>
       </c>
@@ -5708,15 +5708,15 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.73046875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.73046875" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>179</v>
       </c>
@@ -5733,7 +5733,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>192</v>
       </c>
@@ -5750,7 +5750,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>194</v>
       </c>
@@ -5767,7 +5767,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>196</v>
       </c>
@@ -5784,7 +5784,7 @@
         <v>1231</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>197</v>
       </c>
@@ -5801,7 +5801,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>198</v>
       </c>
@@ -5818,7 +5818,7 @@
         <v>1649</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>199</v>
       </c>
@@ -5848,13 +5848,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="5" width="16.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.73046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="5" width="16.73046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>179</v>
       </c>
@@ -5871,7 +5871,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>192</v>
       </c>
@@ -5888,7 +5888,7 @@
         <v>28.012768021347298</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>194</v>
       </c>
@@ -5905,7 +5905,7 @@
         <v>30.438729036495001</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>196</v>
       </c>
@@ -5922,7 +5922,7 @@
         <v>93.253594939231306</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>197</v>
       </c>
@@ -5939,7 +5939,7 @@
         <v>32.969782588859502</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>198</v>
       </c>
@@ -5956,7 +5956,7 @@
         <v>127.911505734532</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>199</v>
       </c>
@@ -5973,7 +5973,7 @@
         <v>14.2977279015767</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>253</v>
       </c>

</xml_diff>